<commit_message>
docs: align traceability docs and refresh submission workbook
</commit_message>
<xml_diff>
--- a/driving-alert-workproducts/excel/submission_final_all_in_one.xlsx
+++ b/driving-alert-workproducts/excel/submission_final_all_in_one.xlsx
@@ -10721,17 +10721,17 @@
     <row r="27">
       <c r="A27" s="2" t="inlineStr">
         <is>
-          <t>30</t>
+          <t>7</t>
         </is>
       </c>
       <c r="B27" s="2" t="inlineStr">
         <is>
-          <t>Infotainment</t>
+          <t>V2X</t>
         </is>
       </c>
       <c r="C27" s="2" t="inlineStr">
         <is>
-          <t>speedLimit</t>
+          <t>emergencyType</t>
         </is>
       </c>
       <c r="D27" s="2" t="inlineStr">
@@ -10746,24 +10746,24 @@
       </c>
       <c r="F27" s="2" t="inlineStr">
         <is>
-          <t>255</t>
+          <t>3</t>
         </is>
       </c>
       <c r="G27" s="2" t="inlineStr">
         <is>
-          <t>30</t>
+          <t>0</t>
         </is>
       </c>
       <c r="H27" s="2" t="inlineStr">
         <is>
-          <t>구간 제한속도(km/h)</t>
+          <t>긴급차량 종류</t>
         </is>
       </c>
     </row>
     <row r="28">
       <c r="A28" s="2" t="inlineStr">
         <is>
-          <t>7</t>
+          <t>8</t>
         </is>
       </c>
       <c r="B28" s="2" t="inlineStr">
@@ -10773,7 +10773,7 @@
       </c>
       <c r="C28" s="2" t="inlineStr">
         <is>
-          <t>emergencyType</t>
+          <t>emergencyDirection</t>
         </is>
       </c>
       <c r="D28" s="2" t="inlineStr">
@@ -10798,14 +10798,14 @@
       </c>
       <c r="H28" s="2" t="inlineStr">
         <is>
-          <t>긴급차량 종류</t>
+          <t>긴급차량 접근 방향</t>
         </is>
       </c>
     </row>
     <row r="29">
       <c r="A29" s="2" t="inlineStr">
         <is>
-          <t>8</t>
+          <t>9</t>
         </is>
       </c>
       <c r="B29" s="2" t="inlineStr">
@@ -10815,7 +10815,7 @@
       </c>
       <c r="C29" s="2" t="inlineStr">
         <is>
-          <t>emergencyDirection</t>
+          <t>EtaSeconds</t>
         </is>
       </c>
       <c r="D29" s="2" t="inlineStr">
@@ -10830,7 +10830,7 @@
       </c>
       <c r="F29" s="2" t="inlineStr">
         <is>
-          <t>3</t>
+          <t>255</t>
         </is>
       </c>
       <c r="G29" s="2" t="inlineStr">
@@ -10840,14 +10840,14 @@
       </c>
       <c r="H29" s="2" t="inlineStr">
         <is>
-          <t>긴급차량 접근 방향</t>
+          <t>긴급차량 ETA(유효값 0~255, 내부 invalid sentinel 65535)</t>
         </is>
       </c>
     </row>
     <row r="30">
       <c r="A30" s="2" t="inlineStr">
         <is>
-          <t>9</t>
+          <t>10</t>
         </is>
       </c>
       <c r="B30" s="2" t="inlineStr">
@@ -10857,7 +10857,7 @@
       </c>
       <c r="C30" s="2" t="inlineStr">
         <is>
-          <t>EtaSeconds</t>
+          <t>SourceId</t>
         </is>
       </c>
       <c r="D30" s="2" t="inlineStr">
@@ -10882,14 +10882,14 @@
       </c>
       <c r="H30" s="2" t="inlineStr">
         <is>
-          <t>긴급차량 ETA(유효값 0~255, 내부 invalid sentinel 65535)</t>
+          <t>긴급 메시지 Source ID</t>
         </is>
       </c>
     </row>
     <row r="31">
       <c r="A31" s="2" t="inlineStr">
         <is>
-          <t>10</t>
+          <t>11</t>
         </is>
       </c>
       <c r="B31" s="2" t="inlineStr">
@@ -10899,7 +10899,7 @@
       </c>
       <c r="C31" s="2" t="inlineStr">
         <is>
-          <t>SourceId</t>
+          <t>Status</t>
         </is>
       </c>
       <c r="D31" s="2" t="inlineStr">
@@ -10914,7 +10914,7 @@
       </c>
       <c r="F31" s="2" t="inlineStr">
         <is>
-          <t>255</t>
+          <t>1</t>
         </is>
       </c>
       <c r="G31" s="2" t="inlineStr">
@@ -10924,24 +10924,24 @@
       </c>
       <c r="H31" s="2" t="inlineStr">
         <is>
-          <t>긴급 메시지 Source ID</t>
+          <t>긴급 메시지 Active/Clear 상태</t>
         </is>
       </c>
     </row>
     <row r="32">
       <c r="A32" s="2" t="inlineStr">
         <is>
-          <t>11</t>
+          <t>12</t>
         </is>
       </c>
       <c r="B32" s="2" t="inlineStr">
         <is>
-          <t>V2X</t>
+          <t>Core</t>
         </is>
       </c>
       <c r="C32" s="2" t="inlineStr">
         <is>
-          <t>Status</t>
+          <t>vehicleSpeedNorm</t>
         </is>
       </c>
       <c r="D32" s="2" t="inlineStr">
@@ -10956,7 +10956,7 @@
       </c>
       <c r="F32" s="2" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>255</t>
         </is>
       </c>
       <c r="G32" s="2" t="inlineStr">
@@ -10966,14 +10966,14 @@
       </c>
       <c r="H32" s="2" t="inlineStr">
         <is>
-          <t>긴급 메시지 Active/Clear 상태</t>
+          <t>게이트웨이 정규화 후 차량 속도</t>
         </is>
       </c>
     </row>
     <row r="33">
       <c r="A33" s="2" t="inlineStr">
         <is>
-          <t>12</t>
+          <t>13</t>
         </is>
       </c>
       <c r="B33" s="2" t="inlineStr">
@@ -10983,7 +10983,7 @@
       </c>
       <c r="C33" s="2" t="inlineStr">
         <is>
-          <t>vehicleSpeedNorm</t>
+          <t>driveStateNorm</t>
         </is>
       </c>
       <c r="D33" s="2" t="inlineStr">
@@ -10998,7 +10998,7 @@
       </c>
       <c r="F33" s="2" t="inlineStr">
         <is>
-          <t>255</t>
+          <t>3</t>
         </is>
       </c>
       <c r="G33" s="2" t="inlineStr">
@@ -11008,14 +11008,14 @@
       </c>
       <c r="H33" s="2" t="inlineStr">
         <is>
-          <t>게이트웨이 정규화 후 차량 속도</t>
+          <t>게이트웨이 정규화 후 주행 상태</t>
         </is>
       </c>
     </row>
     <row r="34">
       <c r="A34" s="2" t="inlineStr">
         <is>
-          <t>13</t>
+          <t>14</t>
         </is>
       </c>
       <c r="B34" s="2" t="inlineStr">
@@ -11025,7 +11025,7 @@
       </c>
       <c r="C34" s="2" t="inlineStr">
         <is>
-          <t>driveStateNorm</t>
+          <t>steeringInputNorm</t>
         </is>
       </c>
       <c r="D34" s="2" t="inlineStr">
@@ -11040,7 +11040,7 @@
       </c>
       <c r="F34" s="2" t="inlineStr">
         <is>
-          <t>3</t>
+          <t>1</t>
         </is>
       </c>
       <c r="G34" s="2" t="inlineStr">
@@ -11050,14 +11050,14 @@
       </c>
       <c r="H34" s="2" t="inlineStr">
         <is>
-          <t>게이트웨이 정규화 후 주행 상태</t>
+          <t>게이트웨이 정규화 후 조향 입력</t>
         </is>
       </c>
     </row>
     <row r="35">
       <c r="A35" s="2" t="inlineStr">
         <is>
-          <t>14</t>
+          <t>15</t>
         </is>
       </c>
       <c r="B35" s="2" t="inlineStr">
@@ -11067,7 +11067,7 @@
       </c>
       <c r="C35" s="2" t="inlineStr">
         <is>
-          <t>steeringInputNorm</t>
+          <t>baseZoneContext</t>
         </is>
       </c>
       <c r="D35" s="2" t="inlineStr">
@@ -11082,7 +11082,7 @@
       </c>
       <c r="F35" s="2" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>255</t>
         </is>
       </c>
       <c r="G35" s="2" t="inlineStr">
@@ -11092,14 +11092,14 @@
       </c>
       <c r="H35" s="2" t="inlineStr">
         <is>
-          <t>게이트웨이 정규화 후 조향 입력</t>
+          <t>구간 컨텍스트 계산 결과</t>
         </is>
       </c>
     </row>
     <row r="36">
       <c r="A36" s="2" t="inlineStr">
         <is>
-          <t>31</t>
+          <t>16</t>
         </is>
       </c>
       <c r="B36" s="2" t="inlineStr">
@@ -11109,7 +11109,7 @@
       </c>
       <c r="C36" s="2" t="inlineStr">
         <is>
-          <t>speedLimitNorm</t>
+          <t>warningState</t>
         </is>
       </c>
       <c r="D36" s="2" t="inlineStr">
@@ -11129,19 +11129,19 @@
       </c>
       <c r="G36" s="2" t="inlineStr">
         <is>
-          <t>30</t>
+          <t>0</t>
         </is>
       </c>
       <c r="H36" s="2" t="inlineStr">
         <is>
-          <t>게이트웨이 정규화 후 구간 제한속도</t>
+          <t>경고 조건 판정 상태</t>
         </is>
       </c>
     </row>
     <row r="37">
       <c r="A37" s="2" t="inlineStr">
         <is>
-          <t>32</t>
+          <t>17</t>
         </is>
       </c>
       <c r="B37" s="2" t="inlineStr">
@@ -11151,7 +11151,7 @@
       </c>
       <c r="C37" s="2" t="inlineStr">
         <is>
-          <t>proximityRiskLevel</t>
+          <t>emergencyContext</t>
         </is>
       </c>
       <c r="D37" s="2" t="inlineStr">
@@ -11166,7 +11166,7 @@
       </c>
       <c r="F37" s="2" t="inlineStr">
         <is>
-          <t>100</t>
+          <t>255</t>
         </is>
       </c>
       <c r="G37" s="2" t="inlineStr">
@@ -11176,14 +11176,14 @@
       </c>
       <c r="H37" s="2" t="inlineStr">
         <is>
-          <t>긴급차량 근접 위험도 산정값</t>
+          <t>긴급 수신 컨텍스트 상태</t>
         </is>
       </c>
     </row>
     <row r="38">
       <c r="A38" s="2" t="inlineStr">
         <is>
-          <t>33</t>
+          <t>18</t>
         </is>
       </c>
       <c r="B38" s="2" t="inlineStr">
@@ -11193,7 +11193,7 @@
       </c>
       <c r="C38" s="2" t="inlineStr">
         <is>
-          <t>decelAssistReq</t>
+          <t>selectedAlertLevel</t>
         </is>
       </c>
       <c r="D38" s="2" t="inlineStr">
@@ -11208,7 +11208,7 @@
       </c>
       <c r="F38" s="2" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>7</t>
         </is>
       </c>
       <c r="G38" s="2" t="inlineStr">
@@ -11218,14 +11218,14 @@
       </c>
       <c r="H38" s="2" t="inlineStr">
         <is>
-          <t>감속 보조 요청 플래그</t>
+          <t>중재 결과 경고 레벨</t>
         </is>
       </c>
     </row>
     <row r="39">
       <c r="A39" s="2" t="inlineStr">
         <is>
-          <t>34</t>
+          <t>19</t>
         </is>
       </c>
       <c r="B39" s="2" t="inlineStr">
@@ -11235,7 +11235,7 @@
       </c>
       <c r="C39" s="2" t="inlineStr">
         <is>
-          <t>failSafeMode</t>
+          <t>selectedAlertType</t>
         </is>
       </c>
       <c r="D39" s="2" t="inlineStr">
@@ -11250,7 +11250,7 @@
       </c>
       <c r="F39" s="2" t="inlineStr">
         <is>
-          <t>2</t>
+          <t>7</t>
         </is>
       </c>
       <c r="G39" s="2" t="inlineStr">
@@ -11260,24 +11260,24 @@
       </c>
       <c r="H39" s="2" t="inlineStr">
         <is>
-          <t>경고 정보 전달 이상 강등 모드</t>
+          <t>중재 결과 경고 타입</t>
         </is>
       </c>
     </row>
     <row r="40">
       <c r="A40" s="2" t="inlineStr">
         <is>
-          <t>35</t>
+          <t>20</t>
         </is>
       </c>
       <c r="B40" s="2" t="inlineStr">
         <is>
-          <t>CoreState</t>
+          <t>Core</t>
         </is>
       </c>
       <c r="C40" s="2" t="inlineStr">
         <is>
-          <t>warningPathStatus</t>
+          <t>timeoutClear</t>
         </is>
       </c>
       <c r="D40" s="2" t="inlineStr">
@@ -11292,7 +11292,7 @@
       </c>
       <c r="F40" s="2" t="inlineStr">
         <is>
-          <t>2</t>
+          <t>1</t>
         </is>
       </c>
       <c r="G40" s="2" t="inlineStr">
@@ -11302,24 +11302,24 @@
       </c>
       <c r="H40" s="2" t="inlineStr">
         <is>
-          <t>경고 정보 전달 경로 상태(정상/열화/단절)</t>
+          <t>1000ms 무갱신 해제 플래그</t>
         </is>
       </c>
     </row>
     <row r="41">
       <c r="A41" s="2" t="inlineStr">
         <is>
-          <t>36</t>
+          <t>21</t>
         </is>
       </c>
       <c r="B41" s="2" t="inlineStr">
         <is>
-          <t>CoreState</t>
+          <t>Body</t>
         </is>
       </c>
       <c r="C41" s="2" t="inlineStr">
         <is>
-          <t>e2eHealthState</t>
+          <t>ambientMode</t>
         </is>
       </c>
       <c r="D41" s="2" t="inlineStr">
@@ -11334,7 +11334,7 @@
       </c>
       <c r="F41" s="2" t="inlineStr">
         <is>
-          <t>2</t>
+          <t>7</t>
         </is>
       </c>
       <c r="G41" s="2" t="inlineStr">
@@ -11344,24 +11344,24 @@
       </c>
       <c r="H41" s="2" t="inlineStr">
         <is>
-          <t>E2E 경로 헬스 상태</t>
+          <t>앰비언트 제어 모드</t>
         </is>
       </c>
     </row>
     <row r="42">
       <c r="A42" s="2" t="inlineStr">
         <is>
-          <t>37</t>
+          <t>22</t>
         </is>
       </c>
       <c r="B42" s="2" t="inlineStr">
         <is>
-          <t>Core</t>
+          <t>Body</t>
         </is>
       </c>
       <c r="C42" s="2" t="inlineStr">
         <is>
-          <t>brakePedalNorm</t>
+          <t>ambientColor</t>
         </is>
       </c>
       <c r="D42" s="2" t="inlineStr">
@@ -11376,7 +11376,7 @@
       </c>
       <c r="F42" s="2" t="inlineStr">
         <is>
-          <t>100</t>
+          <t>7</t>
         </is>
       </c>
       <c r="G42" s="2" t="inlineStr">
@@ -11386,24 +11386,24 @@
       </c>
       <c r="H42" s="2" t="inlineStr">
         <is>
-          <t>CHS_GW에서 정규화한 브레이크 입력</t>
+          <t>앰비언트 색상 코드</t>
         </is>
       </c>
     </row>
     <row r="43">
       <c r="A43" s="2" t="inlineStr">
         <is>
-          <t>38</t>
+          <t>23</t>
         </is>
       </c>
       <c r="B43" s="2" t="inlineStr">
         <is>
-          <t>Test</t>
+          <t>Body</t>
         </is>
       </c>
       <c r="C43" s="2" t="inlineStr">
         <is>
-          <t>forceFailSafe</t>
+          <t>ambientPattern</t>
         </is>
       </c>
       <c r="D43" s="2" t="inlineStr">
@@ -11418,7 +11418,7 @@
       </c>
       <c r="F43" s="2" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>3</t>
         </is>
       </c>
       <c r="G43" s="2" t="inlineStr">
@@ -11428,24 +11428,24 @@
       </c>
       <c r="H43" s="2" t="inlineStr">
         <is>
-          <t>Fail-safe 강제 주입(Validation-only)</t>
+          <t>앰비언트 패턴 코드</t>
         </is>
       </c>
     </row>
     <row r="44">
       <c r="A44" s="2" t="inlineStr">
         <is>
-          <t>49</t>
+          <t>24</t>
         </is>
       </c>
       <c r="B44" s="2" t="inlineStr">
         <is>
-          <t>Test</t>
+          <t>Cluster</t>
         </is>
       </c>
       <c r="C44" s="2" t="inlineStr">
         <is>
-          <t>displayModeSetting</t>
+          <t>warningTextCode</t>
         </is>
       </c>
       <c r="D44" s="2" t="inlineStr">
@@ -11460,7 +11460,7 @@
       </c>
       <c r="F44" s="2" t="inlineStr">
         <is>
-          <t>2</t>
+          <t>255</t>
         </is>
       </c>
       <c r="G44" s="2" t="inlineStr">
@@ -11470,14 +11470,14 @@
       </c>
       <c r="H44" s="2" t="inlineStr">
         <is>
-          <t>표시 모드 수동 설정 입력(Validation-only)</t>
+          <t>클러스터 경고 코드</t>
         </is>
       </c>
     </row>
     <row r="45">
       <c r="A45" s="2" t="inlineStr">
         <is>
-          <t>50</t>
+          <t>25</t>
         </is>
       </c>
       <c r="B45" s="2" t="inlineStr">
@@ -11487,7 +11487,7 @@
       </c>
       <c r="C45" s="2" t="inlineStr">
         <is>
-          <t>alertVolumeSetting</t>
+          <t>testScenario</t>
         </is>
       </c>
       <c r="D45" s="2" t="inlineStr">
@@ -11502,24 +11502,24 @@
       </c>
       <c r="F45" s="2" t="inlineStr">
         <is>
-          <t>100</t>
+          <t>255</t>
         </is>
       </c>
       <c r="G45" s="2" t="inlineStr">
         <is>
-          <t>50</t>
+          <t>0</t>
         </is>
       </c>
       <c r="H45" s="2" t="inlineStr">
         <is>
-          <t>경고 음량 수동 설정 입력(Validation-only)</t>
+          <t>SIL 테스트 시나리오 선택값(Validation-only)</t>
         </is>
       </c>
     </row>
     <row r="46">
       <c r="A46" s="2" t="inlineStr">
         <is>
-          <t>51</t>
+          <t>26</t>
         </is>
       </c>
       <c r="B46" s="2" t="inlineStr">
@@ -11529,7 +11529,7 @@
       </c>
       <c r="C46" s="2" t="inlineStr">
         <is>
-          <t>seatBeltOverride</t>
+          <t>scenarioResult</t>
         </is>
       </c>
       <c r="D46" s="2" t="inlineStr">
@@ -11544,7 +11544,7 @@
       </c>
       <c r="F46" s="2" t="inlineStr">
         <is>
-          <t>2</t>
+          <t>1</t>
         </is>
       </c>
       <c r="G46" s="2" t="inlineStr">
@@ -11554,24 +11554,24 @@
       </c>
       <c r="H46" s="2" t="inlineStr">
         <is>
-          <t>안전벨트 상태 오버라이드 입력(Validation-only)</t>
+          <t>SIL 시나리오 Pass/Fail 결과(Validation-only)</t>
         </is>
       </c>
     </row>
     <row r="47">
       <c r="A47" s="2" t="inlineStr">
         <is>
-          <t>52</t>
+          <t>27</t>
         </is>
       </c>
       <c r="B47" s="2" t="inlineStr">
         <is>
-          <t>Test</t>
+          <t>CoreState</t>
         </is>
       </c>
       <c r="C47" s="2" t="inlineStr">
         <is>
-          <t>historyQueryOffset</t>
+          <t>lastEmergencyRxMs</t>
         </is>
       </c>
       <c r="D47" s="2" t="inlineStr">
@@ -11586,7 +11586,7 @@
       </c>
       <c r="F47" s="2" t="inlineStr">
         <is>
-          <t>255</t>
+          <t>4294967295</t>
         </is>
       </c>
       <c r="G47" s="2" t="inlineStr">
@@ -11596,24 +11596,24 @@
       </c>
       <c r="H47" s="2" t="inlineStr">
         <is>
-          <t>경고 이력 조회 오프셋 입력(Validation-only)</t>
+          <t>마지막 긴급 신호 수신 시각(ms)</t>
         </is>
       </c>
     </row>
     <row r="48">
       <c r="A48" s="2" t="inlineStr">
         <is>
-          <t>53</t>
+          <t>28</t>
         </is>
       </c>
       <c r="B48" s="2" t="inlineStr">
         <is>
-          <t>Test</t>
+          <t>CoreState</t>
         </is>
       </c>
       <c r="C48" s="2" t="inlineStr">
         <is>
-          <t>historyQueryCode</t>
+          <t>duplicatePopupGuard</t>
         </is>
       </c>
       <c r="D48" s="2" t="inlineStr">
@@ -11628,7 +11628,7 @@
       </c>
       <c r="F48" s="2" t="inlineStr">
         <is>
-          <t>65535</t>
+          <t>5000</t>
         </is>
       </c>
       <c r="G48" s="2" t="inlineStr">
@@ -11638,24 +11638,24 @@
       </c>
       <c r="H48" s="2" t="inlineStr">
         <is>
-          <t>경고 이력 조회 코드 입력(Validation-only)</t>
+          <t>중복 팝업 억제 타이머(ms)</t>
         </is>
       </c>
     </row>
     <row r="49">
       <c r="A49" s="2" t="inlineStr">
         <is>
-          <t>39</t>
+          <t>29</t>
         </is>
       </c>
       <c r="B49" s="2" t="inlineStr">
         <is>
-          <t>Core</t>
+          <t>CoreState</t>
         </is>
       </c>
       <c r="C49" s="2" t="inlineStr">
         <is>
-          <t>objectTrackValid</t>
+          <t>arbitrationSnapshotId</t>
         </is>
       </c>
       <c r="D49" s="2" t="inlineStr">
@@ -11670,7 +11670,7 @@
       </c>
       <c r="F49" s="2" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>65535</t>
         </is>
       </c>
       <c r="G49" s="2" t="inlineStr">
@@ -11680,24 +11680,24 @@
       </c>
       <c r="H49" s="2" t="inlineStr">
         <is>
-          <t>객체 추적 유효 플래그</t>
+          <t>중재 스냅샷 식별자</t>
         </is>
       </c>
     </row>
     <row r="50">
       <c r="A50" s="2" t="inlineStr">
         <is>
-          <t>40</t>
+          <t>30</t>
         </is>
       </c>
       <c r="B50" s="2" t="inlineStr">
         <is>
-          <t>Core</t>
+          <t>Infotainment</t>
         </is>
       </c>
       <c r="C50" s="2" t="inlineStr">
         <is>
-          <t>objectRange</t>
+          <t>speedLimit</t>
         </is>
       </c>
       <c r="D50" s="2" t="inlineStr">
@@ -11712,24 +11712,24 @@
       </c>
       <c r="F50" s="2" t="inlineStr">
         <is>
-          <t>500</t>
+          <t>255</t>
         </is>
       </c>
       <c r="G50" s="2" t="inlineStr">
         <is>
-          <t>0</t>
+          <t>30</t>
         </is>
       </c>
       <c r="H50" s="2" t="inlineStr">
         <is>
-          <t>대표 위험 객체 상대 거리(m)</t>
+          <t>구간 제한속도(km/h)</t>
         </is>
       </c>
     </row>
     <row r="51">
       <c r="A51" s="2" t="inlineStr">
         <is>
-          <t>41</t>
+          <t>31</t>
         </is>
       </c>
       <c r="B51" s="2" t="inlineStr">
@@ -11739,39 +11739,39 @@
       </c>
       <c r="C51" s="2" t="inlineStr">
         <is>
-          <t>objectRelSpeed</t>
+          <t>speedLimitNorm</t>
         </is>
       </c>
       <c r="D51" s="2" t="inlineStr">
         <is>
-          <t>int32</t>
+          <t>uint32</t>
         </is>
       </c>
       <c r="E51" s="2" t="inlineStr">
         <is>
-          <t>-200</t>
+          <t>0</t>
         </is>
       </c>
       <c r="F51" s="2" t="inlineStr">
         <is>
-          <t>200</t>
+          <t>255</t>
         </is>
       </c>
       <c r="G51" s="2" t="inlineStr">
         <is>
-          <t>0</t>
+          <t>30</t>
         </is>
       </c>
       <c r="H51" s="2" t="inlineStr">
         <is>
-          <t>대표 위험 객체 상대 속도(km/h)</t>
+          <t>게이트웨이 정규화 후 구간 제한속도</t>
         </is>
       </c>
     </row>
     <row r="52">
       <c r="A52" s="2" t="inlineStr">
         <is>
-          <t>42</t>
+          <t>32</t>
         </is>
       </c>
       <c r="B52" s="2" t="inlineStr">
@@ -11781,7 +11781,7 @@
       </c>
       <c r="C52" s="2" t="inlineStr">
         <is>
-          <t>objectConfidence</t>
+          <t>proximityRiskLevel</t>
         </is>
       </c>
       <c r="D52" s="2" t="inlineStr">
@@ -11806,14 +11806,14 @@
       </c>
       <c r="H52" s="2" t="inlineStr">
         <is>
-          <t>객체 인지 신뢰도(%)</t>
+          <t>긴급차량 근접 위험도 산정값</t>
         </is>
       </c>
     </row>
     <row r="53">
       <c r="A53" s="2" t="inlineStr">
         <is>
-          <t>43</t>
+          <t>33</t>
         </is>
       </c>
       <c r="B53" s="2" t="inlineStr">
@@ -11823,7 +11823,7 @@
       </c>
       <c r="C53" s="2" t="inlineStr">
         <is>
-          <t>objectRiskClass</t>
+          <t>decelAssistReq</t>
         </is>
       </c>
       <c r="D53" s="2" t="inlineStr">
@@ -11838,7 +11838,7 @@
       </c>
       <c r="F53" s="2" t="inlineStr">
         <is>
-          <t>7</t>
+          <t>1</t>
         </is>
       </c>
       <c r="G53" s="2" t="inlineStr">
@@ -11848,14 +11848,14 @@
       </c>
       <c r="H53" s="2" t="inlineStr">
         <is>
-          <t>객체 위험 분류 코드</t>
+          <t>감속 보조 요청 플래그</t>
         </is>
       </c>
     </row>
     <row r="54">
       <c r="A54" s="2" t="inlineStr">
         <is>
-          <t>44</t>
+          <t>34</t>
         </is>
       </c>
       <c r="B54" s="2" t="inlineStr">
@@ -11865,7 +11865,7 @@
       </c>
       <c r="C54" s="2" t="inlineStr">
         <is>
-          <t>objectTtcMin</t>
+          <t>failSafeMode</t>
         </is>
       </c>
       <c r="D54" s="2" t="inlineStr">
@@ -11880,34 +11880,34 @@
       </c>
       <c r="F54" s="2" t="inlineStr">
         <is>
-          <t>10000</t>
+          <t>2</t>
         </is>
       </c>
       <c r="G54" s="2" t="inlineStr">
         <is>
-          <t>10000</t>
+          <t>0</t>
         </is>
       </c>
       <c r="H54" s="2" t="inlineStr">
         <is>
-          <t>대표 위험 객체 최소 TTC(ms)</t>
+          <t>경고 정보 전달 이상 강등 모드</t>
         </is>
       </c>
     </row>
     <row r="55">
       <c r="A55" s="2" t="inlineStr">
         <is>
-          <t>45</t>
+          <t>35</t>
         </is>
       </c>
       <c r="B55" s="2" t="inlineStr">
         <is>
-          <t>Core</t>
+          <t>CoreState</t>
         </is>
       </c>
       <c r="C55" s="2" t="inlineStr">
         <is>
-          <t>intersectionConflictFlag</t>
+          <t>warningPathStatus</t>
         </is>
       </c>
       <c r="D55" s="2" t="inlineStr">
@@ -11922,7 +11922,7 @@
       </c>
       <c r="F55" s="2" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>2</t>
         </is>
       </c>
       <c r="G55" s="2" t="inlineStr">
@@ -11932,24 +11932,24 @@
       </c>
       <c r="H55" s="2" t="inlineStr">
         <is>
-          <t>교차로 측방 접근 충돌 플래그</t>
+          <t>경고 정보 전달 경로 상태(정상/열화/단절)</t>
         </is>
       </c>
     </row>
     <row r="56">
       <c r="A56" s="2" t="inlineStr">
         <is>
-          <t>46</t>
+          <t>36</t>
         </is>
       </c>
       <c r="B56" s="2" t="inlineStr">
         <is>
-          <t>Core</t>
+          <t>CoreState</t>
         </is>
       </c>
       <c r="C56" s="2" t="inlineStr">
         <is>
-          <t>mergeCutInFlag</t>
+          <t>e2eHealthState</t>
         </is>
       </c>
       <c r="D56" s="2" t="inlineStr">
@@ -11964,7 +11964,7 @@
       </c>
       <c r="F56" s="2" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>2</t>
         </is>
       </c>
       <c r="G56" s="2" t="inlineStr">
@@ -11974,14 +11974,14 @@
       </c>
       <c r="H56" s="2" t="inlineStr">
         <is>
-          <t>합류/끼어들기 급간섭 플래그</t>
+          <t>E2E 경로 헬스 상태</t>
         </is>
       </c>
     </row>
     <row r="57">
       <c r="A57" s="2" t="inlineStr">
         <is>
-          <t>47</t>
+          <t>37</t>
         </is>
       </c>
       <c r="B57" s="2" t="inlineStr">
@@ -11991,7 +11991,7 @@
       </c>
       <c r="C57" s="2" t="inlineStr">
         <is>
-          <t>objectAlertHoldMs</t>
+          <t>brakePedalNorm</t>
         </is>
       </c>
       <c r="D57" s="2" t="inlineStr">
@@ -12006,34 +12006,34 @@
       </c>
       <c r="F57" s="2" t="inlineStr">
         <is>
-          <t>5000</t>
+          <t>100</t>
         </is>
       </c>
       <c r="G57" s="2" t="inlineStr">
         <is>
-          <t>300</t>
+          <t>0</t>
         </is>
       </c>
       <c r="H57" s="2" t="inlineStr">
         <is>
-          <t>객체 추적 손실 시 경고 유지시간(ms)</t>
+          <t>CHS_GW에서 정규화한 브레이크 입력</t>
         </is>
       </c>
     </row>
     <row r="58">
       <c r="A58" s="2" t="inlineStr">
         <is>
-          <t>48</t>
+          <t>38</t>
         </is>
       </c>
       <c r="B58" s="2" t="inlineStr">
         <is>
-          <t>Core</t>
+          <t>Test</t>
         </is>
       </c>
       <c r="C58" s="2" t="inlineStr">
         <is>
-          <t>objectEventCode</t>
+          <t>forceFailSafe</t>
         </is>
       </c>
       <c r="D58" s="2" t="inlineStr">
@@ -12048,7 +12048,7 @@
       </c>
       <c r="F58" s="2" t="inlineStr">
         <is>
-          <t>65535</t>
+          <t>1</t>
         </is>
       </c>
       <c r="G58" s="2" t="inlineStr">
@@ -12058,14 +12058,14 @@
       </c>
       <c r="H58" s="2" t="inlineStr">
         <is>
-          <t>객체 기반 경고 이벤트 코드</t>
+          <t>Fail-safe 강제 주입(Validation-only)</t>
         </is>
       </c>
     </row>
     <row r="59">
       <c r="A59" s="2" t="inlineStr">
         <is>
-          <t>15</t>
+          <t>39</t>
         </is>
       </c>
       <c r="B59" s="2" t="inlineStr">
@@ -12075,7 +12075,7 @@
       </c>
       <c r="C59" s="2" t="inlineStr">
         <is>
-          <t>baseZoneContext</t>
+          <t>objectTrackValid</t>
         </is>
       </c>
       <c r="D59" s="2" t="inlineStr">
@@ -12090,7 +12090,7 @@
       </c>
       <c r="F59" s="2" t="inlineStr">
         <is>
-          <t>255</t>
+          <t>1</t>
         </is>
       </c>
       <c r="G59" s="2" t="inlineStr">
@@ -12100,14 +12100,14 @@
       </c>
       <c r="H59" s="2" t="inlineStr">
         <is>
-          <t>구간 컨텍스트 계산 결과</t>
+          <t>객체 추적 유효 플래그</t>
         </is>
       </c>
     </row>
     <row r="60">
       <c r="A60" s="2" t="inlineStr">
         <is>
-          <t>16</t>
+          <t>40</t>
         </is>
       </c>
       <c r="B60" s="2" t="inlineStr">
@@ -12117,7 +12117,7 @@
       </c>
       <c r="C60" s="2" t="inlineStr">
         <is>
-          <t>warningState</t>
+          <t>objectRange</t>
         </is>
       </c>
       <c r="D60" s="2" t="inlineStr">
@@ -12132,7 +12132,7 @@
       </c>
       <c r="F60" s="2" t="inlineStr">
         <is>
-          <t>255</t>
+          <t>500</t>
         </is>
       </c>
       <c r="G60" s="2" t="inlineStr">
@@ -12142,14 +12142,14 @@
       </c>
       <c r="H60" s="2" t="inlineStr">
         <is>
-          <t>경고 조건 판정 상태</t>
+          <t>대표 위험 객체 상대 거리(m)</t>
         </is>
       </c>
     </row>
     <row r="61">
       <c r="A61" s="2" t="inlineStr">
         <is>
-          <t>17</t>
+          <t>41</t>
         </is>
       </c>
       <c r="B61" s="2" t="inlineStr">
@@ -12159,22 +12159,22 @@
       </c>
       <c r="C61" s="2" t="inlineStr">
         <is>
-          <t>emergencyContext</t>
+          <t>objectRelSpeed</t>
         </is>
       </c>
       <c r="D61" s="2" t="inlineStr">
         <is>
-          <t>uint32</t>
+          <t>int32</t>
         </is>
       </c>
       <c r="E61" s="2" t="inlineStr">
         <is>
-          <t>0</t>
+          <t>-200</t>
         </is>
       </c>
       <c r="F61" s="2" t="inlineStr">
         <is>
-          <t>255</t>
+          <t>200</t>
         </is>
       </c>
       <c r="G61" s="2" t="inlineStr">
@@ -12184,14 +12184,14 @@
       </c>
       <c r="H61" s="2" t="inlineStr">
         <is>
-          <t>긴급 수신 컨텍스트 상태</t>
+          <t>대표 위험 객체 상대 속도(km/h)</t>
         </is>
       </c>
     </row>
     <row r="62">
       <c r="A62" s="2" t="inlineStr">
         <is>
-          <t>18</t>
+          <t>42</t>
         </is>
       </c>
       <c r="B62" s="2" t="inlineStr">
@@ -12201,7 +12201,7 @@
       </c>
       <c r="C62" s="2" t="inlineStr">
         <is>
-          <t>selectedAlertLevel</t>
+          <t>objectConfidence</t>
         </is>
       </c>
       <c r="D62" s="2" t="inlineStr">
@@ -12216,7 +12216,7 @@
       </c>
       <c r="F62" s="2" t="inlineStr">
         <is>
-          <t>7</t>
+          <t>100</t>
         </is>
       </c>
       <c r="G62" s="2" t="inlineStr">
@@ -12226,14 +12226,14 @@
       </c>
       <c r="H62" s="2" t="inlineStr">
         <is>
-          <t>중재 결과 경고 레벨</t>
+          <t>객체 인지 신뢰도(%)</t>
         </is>
       </c>
     </row>
     <row r="63">
       <c r="A63" s="2" t="inlineStr">
         <is>
-          <t>19</t>
+          <t>43</t>
         </is>
       </c>
       <c r="B63" s="2" t="inlineStr">
@@ -12243,7 +12243,7 @@
       </c>
       <c r="C63" s="2" t="inlineStr">
         <is>
-          <t>selectedAlertType</t>
+          <t>objectRiskClass</t>
         </is>
       </c>
       <c r="D63" s="2" t="inlineStr">
@@ -12268,14 +12268,14 @@
       </c>
       <c r="H63" s="2" t="inlineStr">
         <is>
-          <t>중재 결과 경고 타입</t>
+          <t>객체 위험 분류 코드</t>
         </is>
       </c>
     </row>
     <row r="64">
       <c r="A64" s="2" t="inlineStr">
         <is>
-          <t>20</t>
+          <t>44</t>
         </is>
       </c>
       <c r="B64" s="2" t="inlineStr">
@@ -12285,7 +12285,7 @@
       </c>
       <c r="C64" s="2" t="inlineStr">
         <is>
-          <t>timeoutClear</t>
+          <t>objectTtcMin</t>
         </is>
       </c>
       <c r="D64" s="2" t="inlineStr">
@@ -12300,34 +12300,34 @@
       </c>
       <c r="F64" s="2" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>10000</t>
         </is>
       </c>
       <c r="G64" s="2" t="inlineStr">
         <is>
-          <t>0</t>
+          <t>10000</t>
         </is>
       </c>
       <c r="H64" s="2" t="inlineStr">
         <is>
-          <t>1000ms 무갱신 해제 플래그</t>
+          <t>대표 위험 객체 최소 TTC(ms)</t>
         </is>
       </c>
     </row>
     <row r="65">
       <c r="A65" s="2" t="inlineStr">
         <is>
-          <t>21</t>
+          <t>45</t>
         </is>
       </c>
       <c r="B65" s="2" t="inlineStr">
         <is>
-          <t>Body</t>
+          <t>Core</t>
         </is>
       </c>
       <c r="C65" s="2" t="inlineStr">
         <is>
-          <t>ambientMode</t>
+          <t>intersectionConflictFlag</t>
         </is>
       </c>
       <c r="D65" s="2" t="inlineStr">
@@ -12342,7 +12342,7 @@
       </c>
       <c r="F65" s="2" t="inlineStr">
         <is>
-          <t>7</t>
+          <t>1</t>
         </is>
       </c>
       <c r="G65" s="2" t="inlineStr">
@@ -12352,24 +12352,24 @@
       </c>
       <c r="H65" s="2" t="inlineStr">
         <is>
-          <t>앰비언트 제어 모드</t>
+          <t>교차로 측방 접근 충돌 플래그</t>
         </is>
       </c>
     </row>
     <row r="66">
       <c r="A66" s="2" t="inlineStr">
         <is>
-          <t>22</t>
+          <t>46</t>
         </is>
       </c>
       <c r="B66" s="2" t="inlineStr">
         <is>
-          <t>Body</t>
+          <t>Core</t>
         </is>
       </c>
       <c r="C66" s="2" t="inlineStr">
         <is>
-          <t>ambientColor</t>
+          <t>mergeCutInFlag</t>
         </is>
       </c>
       <c r="D66" s="2" t="inlineStr">
@@ -12384,7 +12384,7 @@
       </c>
       <c r="F66" s="2" t="inlineStr">
         <is>
-          <t>7</t>
+          <t>1</t>
         </is>
       </c>
       <c r="G66" s="2" t="inlineStr">
@@ -12394,24 +12394,24 @@
       </c>
       <c r="H66" s="2" t="inlineStr">
         <is>
-          <t>앰비언트 색상 코드</t>
+          <t>합류/끼어들기 급간섭 플래그</t>
         </is>
       </c>
     </row>
     <row r="67">
       <c r="A67" s="2" t="inlineStr">
         <is>
-          <t>23</t>
+          <t>47</t>
         </is>
       </c>
       <c r="B67" s="2" t="inlineStr">
         <is>
-          <t>Body</t>
+          <t>Core</t>
         </is>
       </c>
       <c r="C67" s="2" t="inlineStr">
         <is>
-          <t>ambientPattern</t>
+          <t>objectAlertHoldMs</t>
         </is>
       </c>
       <c r="D67" s="2" t="inlineStr">
@@ -12426,34 +12426,34 @@
       </c>
       <c r="F67" s="2" t="inlineStr">
         <is>
-          <t>3</t>
+          <t>5000</t>
         </is>
       </c>
       <c r="G67" s="2" t="inlineStr">
         <is>
-          <t>0</t>
+          <t>300</t>
         </is>
       </c>
       <c r="H67" s="2" t="inlineStr">
         <is>
-          <t>앰비언트 패턴 코드</t>
+          <t>객체 추적 손실 시 경고 유지시간(ms)</t>
         </is>
       </c>
     </row>
     <row r="68">
       <c r="A68" s="2" t="inlineStr">
         <is>
-          <t>24</t>
+          <t>48</t>
         </is>
       </c>
       <c r="B68" s="2" t="inlineStr">
         <is>
-          <t>Cluster</t>
+          <t>Core</t>
         </is>
       </c>
       <c r="C68" s="2" t="inlineStr">
         <is>
-          <t>warningTextCode</t>
+          <t>objectEventCode</t>
         </is>
       </c>
       <c r="D68" s="2" t="inlineStr">
@@ -12468,7 +12468,7 @@
       </c>
       <c r="F68" s="2" t="inlineStr">
         <is>
-          <t>255</t>
+          <t>65535</t>
         </is>
       </c>
       <c r="G68" s="2" t="inlineStr">
@@ -12478,14 +12478,14 @@
       </c>
       <c r="H68" s="2" t="inlineStr">
         <is>
-          <t>클러스터 경고 코드</t>
+          <t>객체 기반 경고 이벤트 코드</t>
         </is>
       </c>
     </row>
     <row r="69">
       <c r="A69" s="2" t="inlineStr">
         <is>
-          <t>25</t>
+          <t>49</t>
         </is>
       </c>
       <c r="B69" s="2" t="inlineStr">
@@ -12495,7 +12495,7 @@
       </c>
       <c r="C69" s="2" t="inlineStr">
         <is>
-          <t>testScenario</t>
+          <t>displayModeSetting</t>
         </is>
       </c>
       <c r="D69" s="2" t="inlineStr">
@@ -12510,7 +12510,7 @@
       </c>
       <c r="F69" s="2" t="inlineStr">
         <is>
-          <t>255</t>
+          <t>2</t>
         </is>
       </c>
       <c r="G69" s="2" t="inlineStr">
@@ -12520,14 +12520,14 @@
       </c>
       <c r="H69" s="2" t="inlineStr">
         <is>
-          <t>SIL 테스트 시나리오 선택값(Validation-only)</t>
+          <t>표시 모드 수동 설정 입력(Validation-only)</t>
         </is>
       </c>
     </row>
     <row r="70">
       <c r="A70" s="2" t="inlineStr">
         <is>
-          <t>26</t>
+          <t>50</t>
         </is>
       </c>
       <c r="B70" s="2" t="inlineStr">
@@ -12537,7 +12537,7 @@
       </c>
       <c r="C70" s="2" t="inlineStr">
         <is>
-          <t>scenarioResult</t>
+          <t>alertVolumeSetting</t>
         </is>
       </c>
       <c r="D70" s="2" t="inlineStr">
@@ -12552,34 +12552,34 @@
       </c>
       <c r="F70" s="2" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>100</t>
         </is>
       </c>
       <c r="G70" s="2" t="inlineStr">
         <is>
-          <t>0</t>
+          <t>50</t>
         </is>
       </c>
       <c r="H70" s="2" t="inlineStr">
         <is>
-          <t>SIL 시나리오 Pass/Fail 결과(Validation-only)</t>
+          <t>경고 음량 수동 설정 입력(Validation-only)</t>
         </is>
       </c>
     </row>
     <row r="71">
       <c r="A71" s="2" t="inlineStr">
         <is>
-          <t>27</t>
+          <t>51</t>
         </is>
       </c>
       <c r="B71" s="2" t="inlineStr">
         <is>
-          <t>CoreState</t>
+          <t>Test</t>
         </is>
       </c>
       <c r="C71" s="2" t="inlineStr">
         <is>
-          <t>lastEmergencyRxMs</t>
+          <t>seatBeltOverride</t>
         </is>
       </c>
       <c r="D71" s="2" t="inlineStr">
@@ -12594,7 +12594,7 @@
       </c>
       <c r="F71" s="2" t="inlineStr">
         <is>
-          <t>4294967295</t>
+          <t>2</t>
         </is>
       </c>
       <c r="G71" s="2" t="inlineStr">
@@ -12604,24 +12604,24 @@
       </c>
       <c r="H71" s="2" t="inlineStr">
         <is>
-          <t>마지막 긴급 신호 수신 시각(ms)</t>
+          <t>안전벨트 상태 오버라이드 입력(Validation-only)</t>
         </is>
       </c>
     </row>
     <row r="72">
       <c r="A72" s="2" t="inlineStr">
         <is>
-          <t>28</t>
+          <t>52</t>
         </is>
       </c>
       <c r="B72" s="2" t="inlineStr">
         <is>
-          <t>CoreState</t>
+          <t>Test</t>
         </is>
       </c>
       <c r="C72" s="2" t="inlineStr">
         <is>
-          <t>duplicatePopupGuard</t>
+          <t>historyQueryOffset</t>
         </is>
       </c>
       <c r="D72" s="2" t="inlineStr">
@@ -12636,7 +12636,7 @@
       </c>
       <c r="F72" s="2" t="inlineStr">
         <is>
-          <t>5000</t>
+          <t>255</t>
         </is>
       </c>
       <c r="G72" s="2" t="inlineStr">
@@ -12646,24 +12646,24 @@
       </c>
       <c r="H72" s="2" t="inlineStr">
         <is>
-          <t>중복 팝업 억제 타이머(ms)</t>
+          <t>경고 이력 조회 오프셋 입력(Validation-only)</t>
         </is>
       </c>
     </row>
     <row r="73">
       <c r="A73" s="2" t="inlineStr">
         <is>
-          <t>29</t>
+          <t>53</t>
         </is>
       </c>
       <c r="B73" s="2" t="inlineStr">
         <is>
-          <t>CoreState</t>
+          <t>Test</t>
         </is>
       </c>
       <c r="C73" s="2" t="inlineStr">
         <is>
-          <t>arbitrationSnapshotId</t>
+          <t>historyQueryCode</t>
         </is>
       </c>
       <c r="D73" s="2" t="inlineStr">
@@ -12688,7 +12688,7 @@
       </c>
       <c r="H73" s="2" t="inlineStr">
         <is>
-          <t>중재 스냅샷 식별자</t>
+          <t>경고 이력 조회 코드 입력(Validation-only)</t>
         </is>
       </c>
     </row>
@@ -22216,12 +22216,12 @@
       <c r="B23" s="2" t="inlineStr"/>
       <c r="C23" s="2" t="inlineStr">
         <is>
-          <t>UT_009 - IVI (NAV_CTX_MGR)</t>
+          <t>UT_003 - ADAS (ADAS_WARN_CTRL)</t>
         </is>
       </c>
       <c r="D23" s="2" t="inlineStr">
         <is>
-          <t>구간, 방향, 거리, 제한속도 정보를 받아 주행 맥락을 계산</t>
+          <t>주행 상태와 제한속도(km/h)를 반영하여 150ms 이내 기본 경고 상태를 판단</t>
         </is>
       </c>
       <c r="E23" s="2" t="inlineStr"/>
@@ -22233,15 +22233,19 @@
       <c r="B24" s="2" t="inlineStr"/>
       <c r="C24" s="2" t="inlineStr">
         <is>
-          <t>UT_003 - ADAS (ADAS_WARN_CTRL)</t>
+          <t>UT_004 - V2X (EMS_ALERT, V2 확장)</t>
         </is>
       </c>
       <c r="D24" s="2" t="inlineStr">
         <is>
-          <t>주행 상태와 제한속도(km/h)를 반영하여 150ms 이내 기본 경고 상태를 판단</t>
-        </is>
-      </c>
-      <c r="E24" s="2" t="inlineStr"/>
+          <t>긴급차량 접근 정보를 수신하고 1000ms 기준 유지, 해제, 타임아웃을 관리</t>
+        </is>
+      </c>
+      <c r="E24" s="2" t="inlineStr">
+        <is>
+          <t>Ready</t>
+        </is>
+      </c>
       <c r="F24" s="2" t="inlineStr"/>
       <c r="G24" s="2" t="inlineStr"/>
     </row>
@@ -22250,15 +22254,19 @@
       <c r="B25" s="2" t="inlineStr"/>
       <c r="C25" s="2" t="inlineStr">
         <is>
-          <t>UT_010 - V2X (EMS_ALERT)</t>
+          <t>UT_005 - ADAS (WARN_ARB_MGR, V2 확장)</t>
         </is>
       </c>
       <c r="D25" s="2" t="inlineStr">
         <is>
-          <t>경찰, 구급 긴급 이벤트의 송신, 수신, 해제, 1000ms 타임아웃 동작을 검증</t>
-        </is>
-      </c>
-      <c r="E25" s="2" t="inlineStr"/>
+          <t>긴급차량 방향과 접근 시간을 반영하여 위험도와 감속 보조를 판단</t>
+        </is>
+      </c>
+      <c r="E25" s="2" t="inlineStr">
+        <is>
+          <t>Ready</t>
+        </is>
+      </c>
       <c r="F25" s="2" t="inlineStr"/>
       <c r="G25" s="2" t="inlineStr"/>
     </row>
@@ -22267,15 +22275,19 @@
       <c r="B26" s="2" t="inlineStr"/>
       <c r="C26" s="2" t="inlineStr">
         <is>
-          <t>UT_011 - ADAS (WARN_ARB_MGR)</t>
+          <t>UT_006 - ADAS (ADAS_WARN_CTRL, ADAS 객체 확장, Planned)</t>
         </is>
       </c>
       <c r="D26" s="2" t="inlineStr">
         <is>
-          <t>긴급 경고와 일반 경고가 겹칠 때 우선순위를 결정</t>
-        </is>
-      </c>
-      <c r="E26" s="2" t="inlineStr"/>
+          <t>주변 객체와 센서 상태를 반영하여 위험 경고를 판단</t>
+        </is>
+      </c>
+      <c r="E26" s="2" t="inlineStr">
+        <is>
+          <t>Planned</t>
+        </is>
+      </c>
       <c r="F26" s="2" t="inlineStr"/>
       <c r="G26" s="2" t="inlineStr"/>
     </row>
@@ -22284,15 +22296,19 @@
       <c r="B27" s="2" t="inlineStr"/>
       <c r="C27" s="2" t="inlineStr">
         <is>
-          <t>UT_012 - BCM (BODY_GW)</t>
+          <t>UT_007 - CLU (CLU_HMI_CTRL, 차량 경보 편의 확장, Planned)</t>
         </is>
       </c>
       <c r="D27" s="2" t="inlineStr">
         <is>
-          <t>경고 결과를 50ms 주기로 앰비언트 출력 경로에 전달</t>
-        </is>
-      </c>
-      <c r="E27" s="2" t="inlineStr"/>
+          <t>운전자 상태와 차량 맥락을 반영하여 경고 표시와 안내를 보정</t>
+        </is>
+      </c>
+      <c r="E27" s="2" t="inlineStr">
+        <is>
+          <t>Planned</t>
+        </is>
+      </c>
       <c r="F27" s="2" t="inlineStr"/>
       <c r="G27" s="2" t="inlineStr"/>
     </row>
@@ -22301,15 +22317,19 @@
       <c r="B28" s="2" t="inlineStr"/>
       <c r="C28" s="2" t="inlineStr">
         <is>
-          <t>UT_013 - IVI (IVI_GW)</t>
+          <t>UT_008 - CGW (DOMAIN_BOUNDARY_MGR, 경고 강건성·인지성 확장, Planned)</t>
         </is>
       </c>
       <c r="D28" s="2" t="inlineStr">
         <is>
-          <t>경고 결과를 50ms 주기로 클러스터 표시 경로에 전달</t>
-        </is>
-      </c>
-      <c r="E28" s="2" t="inlineStr"/>
+          <t>입력 신선도와 서비스 상태를 반영하여 경고 강등과 경계 상태를 유지</t>
+        </is>
+      </c>
+      <c r="E28" s="2" t="inlineStr">
+        <is>
+          <t>Planned</t>
+        </is>
+      </c>
       <c r="F28" s="2" t="inlineStr"/>
       <c r="G28" s="2" t="inlineStr"/>
     </row>
@@ -22318,12 +22338,12 @@
       <c r="B29" s="2" t="inlineStr"/>
       <c r="C29" s="2" t="inlineStr">
         <is>
-          <t>UT_014 - BCM (AMBIENT_CTRL)</t>
+          <t>UT_009 - IVI (NAV_CTX_MGR)</t>
         </is>
       </c>
       <c r="D29" s="2" t="inlineStr">
         <is>
-          <t>경고 상태에 맞는 앰비언트 색상과 패턴을 50ms 주기로 출력</t>
+          <t>구간, 방향, 거리, 제한속도 정보를 받아 주행 맥락을 계산</t>
         </is>
       </c>
       <c r="E29" s="2" t="inlineStr"/>
@@ -22335,12 +22355,12 @@
       <c r="B30" s="2" t="inlineStr"/>
       <c r="C30" s="2" t="inlineStr">
         <is>
-          <t>UT_015 - CLU (CLU_HMI_CTRL)</t>
+          <t>UT_010 - V2X (EMS_ALERT)</t>
         </is>
       </c>
       <c r="D30" s="2" t="inlineStr">
         <is>
-          <t>경고 문구와 방향 표시를 50ms 주기로 출력</t>
+          <t>경찰, 구급 긴급 이벤트의 송신, 수신, 해제, 1000ms 타임아웃 동작을 검증</t>
         </is>
       </c>
       <c r="E30" s="2" t="inlineStr"/>
@@ -22352,19 +22372,15 @@
       <c r="B31" s="2" t="inlineStr"/>
       <c r="C31" s="2" t="inlineStr">
         <is>
-          <t>UT_004 - V2X (EMS_ALERT, V2 확장)</t>
+          <t>UT_011 - ADAS (WARN_ARB_MGR)</t>
         </is>
       </c>
       <c r="D31" s="2" t="inlineStr">
         <is>
-          <t>긴급차량 접근 정보를 수신하고 1000ms 기준 유지, 해제, 타임아웃을 관리</t>
-        </is>
-      </c>
-      <c r="E31" s="2" t="inlineStr">
-        <is>
-          <t>Ready</t>
-        </is>
-      </c>
+          <t>긴급 경고와 일반 경고가 겹칠 때 우선순위를 결정</t>
+        </is>
+      </c>
+      <c r="E31" s="2" t="inlineStr"/>
       <c r="F31" s="2" t="inlineStr"/>
       <c r="G31" s="2" t="inlineStr"/>
     </row>
@@ -22373,19 +22389,15 @@
       <c r="B32" s="2" t="inlineStr"/>
       <c r="C32" s="2" t="inlineStr">
         <is>
-          <t>UT_005 - ADAS (WARN_ARB_MGR, V2 확장)</t>
+          <t>UT_012 - BCM (BODY_GW)</t>
         </is>
       </c>
       <c r="D32" s="2" t="inlineStr">
         <is>
-          <t>긴급차량 방향과 접근 시간을 반영하여 위험도와 감속 보조를 판단</t>
-        </is>
-      </c>
-      <c r="E32" s="2" t="inlineStr">
-        <is>
-          <t>Ready</t>
-        </is>
-      </c>
+          <t>경고 결과를 50ms 주기로 앰비언트 출력 경로에 전달</t>
+        </is>
+      </c>
+      <c r="E32" s="2" t="inlineStr"/>
       <c r="F32" s="2" t="inlineStr"/>
       <c r="G32" s="2" t="inlineStr"/>
     </row>
@@ -22394,19 +22406,15 @@
       <c r="B33" s="2" t="inlineStr"/>
       <c r="C33" s="2" t="inlineStr">
         <is>
-          <t>UT_008 - CGW (DOMAIN_BOUNDARY_MGR, 경고 강건성·인지성 확장, Planned)</t>
+          <t>UT_013 - IVI (IVI_GW)</t>
         </is>
       </c>
       <c r="D33" s="2" t="inlineStr">
         <is>
-          <t>입력 신선도와 서비스 상태를 반영하여 경고 강등과 경계 상태를 유지</t>
-        </is>
-      </c>
-      <c r="E33" s="2" t="inlineStr">
-        <is>
-          <t>Planned</t>
-        </is>
-      </c>
+          <t>경고 결과를 50ms 주기로 클러스터 표시 경로에 전달</t>
+        </is>
+      </c>
+      <c r="E33" s="2" t="inlineStr"/>
       <c r="F33" s="2" t="inlineStr"/>
       <c r="G33" s="2" t="inlineStr"/>
     </row>
@@ -22415,19 +22423,15 @@
       <c r="B34" s="2" t="inlineStr"/>
       <c r="C34" s="2" t="inlineStr">
         <is>
-          <t>UT_006 - ADAS (ADAS_WARN_CTRL, ADAS 객체 확장, Planned)</t>
+          <t>UT_014 - BCM (AMBIENT_CTRL)</t>
         </is>
       </c>
       <c r="D34" s="2" t="inlineStr">
         <is>
-          <t>주변 객체와 센서 상태를 반영하여 위험 경고를 판단</t>
-        </is>
-      </c>
-      <c r="E34" s="2" t="inlineStr">
-        <is>
-          <t>Planned</t>
-        </is>
-      </c>
+          <t>경고 상태에 맞는 앰비언트 색상과 패턴을 50ms 주기로 출력</t>
+        </is>
+      </c>
+      <c r="E34" s="2" t="inlineStr"/>
       <c r="F34" s="2" t="inlineStr"/>
       <c r="G34" s="2" t="inlineStr"/>
     </row>
@@ -22436,19 +22440,15 @@
       <c r="B35" s="2" t="inlineStr"/>
       <c r="C35" s="2" t="inlineStr">
         <is>
-          <t>UT_007 - CLU (CLU_HMI_CTRL, 차량 경보 편의 확장, Planned)</t>
+          <t>UT_015 - CLU (CLU_HMI_CTRL)</t>
         </is>
       </c>
       <c r="D35" s="2" t="inlineStr">
         <is>
-          <t>운전자 상태와 차량 맥락을 반영하여 경고 표시와 안내를 보정</t>
-        </is>
-      </c>
-      <c r="E35" s="2" t="inlineStr">
-        <is>
-          <t>Planned</t>
-        </is>
-      </c>
+          <t>경고 문구와 방향 표시를 50ms 주기로 출력</t>
+        </is>
+      </c>
+      <c r="E35" s="2" t="inlineStr"/>
       <c r="F35" s="2" t="inlineStr"/>
       <c r="G35" s="2" t="inlineStr"/>
     </row>
@@ -23645,7 +23645,7 @@
   <cols>
     <col width="48" customWidth="1" min="1" max="1"/>
     <col width="48" customWidth="1" min="2" max="2"/>
-    <col width="46" customWidth="1" min="3" max="3"/>
+    <col width="48" customWidth="1" min="3" max="3"/>
     <col width="48" customWidth="1" min="4" max="4"/>
     <col width="12" customWidth="1" min="5" max="5"/>
     <col width="12" customWidth="1" min="6" max="6"/>
@@ -24119,7 +24119,7 @@
       </c>
       <c r="B28" s="2" t="inlineStr">
         <is>
-          <t>Req_005,Req_019,Req_020,Req_021,Req_026,Req_033,Req_034,Req_036</t>
+          <t>Req_005,Req_018,Req_019,Req_020,Req_021,Req_026,Req_036</t>
         </is>
       </c>
       <c r="C28" s="2" t="inlineStr">
@@ -24129,7 +24129,7 @@
       </c>
       <c r="D28" s="2" t="inlineStr">
         <is>
-          <t>경고 문구, 방향 정보, 복귀 동작이 클러스터 안내와 일치하고 경고 전환 시 반복 토글 없이 안정적으로 표시된다</t>
+          <t>경고 문구, 긴급차량 종류, 방향 정보가 클러스터 안내와 일치하고 경고 전환 시 반복 토글 없이 안정적으로 표시된다</t>
         </is>
       </c>
       <c r="E28" s="2" t="inlineStr"/>
@@ -24144,17 +24144,17 @@
       </c>
       <c r="B29" s="2" t="inlineStr">
         <is>
-          <t>Req_023,Req_032,Req_033</t>
+          <t>Req_022,Req_023,Req_025,Req_032,Req_076,Req_077</t>
         </is>
       </c>
       <c r="C29" s="2" t="inlineStr">
         <is>
-          <t>긴급 알림 미수신 시 안전 해제와 복귀 통합 검증</t>
+          <t>긴급 종료 신호 및 미수신 시 안전 해제와 복귀 통합 검증</t>
         </is>
       </c>
       <c r="D29" s="2" t="inlineStr">
         <is>
-          <t>1000ms 동안 갱신이 없으면 경고가 안전하게 해제되고 150ms 이내 기본 상태로 복귀하며 중복 토글이 없다</t>
+          <t>종료 신호 수신 또는 1000ms 동안 갱신이 없으면 stale 보호 정책이 적용되고 경고가 안전하게 해제되며 직전 유효 구간 경고 또는 기본 상태로 150ms 이내 복귀하고 중복 표시와 반복 토글이 없다</t>
         </is>
       </c>
       <c r="E29" s="2" t="inlineStr"/>
@@ -24227,17 +24227,17 @@
       </c>
       <c r="B32" s="2" t="inlineStr">
         <is>
-          <t>Req_057,Req_058,Req_059,Req_060,Req_061,Req_062,Req_063,Req_064,Req_065,Req_066</t>
+          <t>Req_057,Req_058,Req_059,Req_060,Req_061,Req_062,Req_063,Req_064,Req_065,Req_075</t>
         </is>
       </c>
       <c r="C32" s="2" t="inlineStr">
         <is>
-          <t>객체 위험 판단 및 이벤트 기록 통합 검증</t>
+          <t>객체 위험 판단, 입력 유효성 필터링 및 이벤트 기록 통합 검증</t>
         </is>
       </c>
       <c r="D32" s="2" t="inlineStr">
         <is>
-          <t>객체 입력은 100ms 이내 반영되고 위험 경고는 150ms 이내 발생하며 신뢰도 저하 시 강등과 이벤트 기록이 누락 없이 수행된다</t>
+          <t>객체 입력은 100ms 이내 반영되고 유효성 미달 입력은 경고 판정에서 제외되며 위험 경고는 150ms 이내 발생하고 신뢰도 저하 시 강등과 이벤트 기록이 누락 없이 수행된다</t>
         </is>
       </c>
       <c r="E32" s="2" t="inlineStr">
@@ -24256,17 +24256,17 @@
       </c>
       <c r="B33" s="2" t="inlineStr">
         <is>
-          <t>Req_067,Req_068,Req_069,Req_070,Req_071,Req_072,Req_073,Req_074</t>
+          <t>Req_067,Req_068,Req_069,Req_073,Req_074</t>
         </is>
       </c>
       <c r="C33" s="2" t="inlineStr">
         <is>
-          <t>운전자 상태, 경고 설정, 접근거리 표시 반영 통합 검증</t>
+          <t>운전자 상태와 경고 설정 반영 통합 검증</t>
         </is>
       </c>
       <c r="D33" s="2" t="inlineStr">
         <is>
-          <t>입력 보정은 150ms 이내 반영되고 접근거리 표시는 200ms 이내 갱신되며 표시·음량 설정은 150ms 이내 반영된다</t>
+          <t>방향지시등, 주행모드, 안전벨트 상태 기반 보정이 150ms 이내 반영되고 표시 방식 및 음량 설정이 150ms 이내 출력 정책에 반영된다</t>
         </is>
       </c>
       <c r="E33" s="2" t="inlineStr">
@@ -24285,17 +24285,17 @@
       </c>
       <c r="B34" s="2" t="inlineStr">
         <is>
-          <t>Req_049,Req_050,Req_057,Req_058,Req_059,Req_060,Req_061,Req_062,Req_063</t>
+          <t>Req_049,Req_050,Req_057,Req_058,Req_059,Req_060,Req_061,Req_062,Req_063,Req_066</t>
         </is>
       </c>
       <c r="C34" s="2" t="inlineStr">
         <is>
-          <t>긴급차량 접근과 교차로/합류 TTC 충돌 위험 동시 입력 통합 검증</t>
+          <t>긴급차량 접근과 교차로/합류 TTC 충돌 위험 동시 입력 시 우선 경고 선택 통합 검증</t>
         </is>
       </c>
       <c r="D34" s="2" t="inlineStr">
         <is>
-          <t>긴급차량이 교차로 또는 합류 구간에서 접근하고 TTC 충돌 위험이 기준 이상이면 자동 감속 보조 요청이 생성되며 우선 경고 선택과 표시 채널 출력이 상충 없이 유지된다</t>
+          <t>긴급차량이 교차로 또는 합류 구간에서 접근하고 TTC 충돌 위험이 기준 이상이면 자동 감속 보조 요청이 생성되며 최종 경고가 우선순위 규칙에 따라 단일 선택되고 표시 채널 출력이 상충 없이 유지된다</t>
         </is>
       </c>
       <c r="E34" s="2" t="inlineStr">
@@ -24319,12 +24319,12 @@
       </c>
       <c r="C35" s="2" t="inlineStr">
         <is>
-          <t>엔진, 변속, 동력 상태 통합 검증</t>
+          <t>시동·기어 상태 통합 검증</t>
         </is>
       </c>
       <c r="D35" s="2" t="inlineStr">
         <is>
-          <t>엔진, 변속, 동력 상태가 100ms 주기로 일관되게 반영된다</t>
+          <t>시동과 기어 상태가 100ms 주기로 일관되게 반영된다</t>
         </is>
       </c>
       <c r="E35" s="2" t="inlineStr"/>
@@ -24344,12 +24344,12 @@
       </c>
       <c r="C36" s="2" t="inlineStr">
         <is>
-          <t>가감속, 조향, 제동, 차체 상태 통합 검증</t>
+          <t>가속, 제동, 조향 입력 통합 검증</t>
         </is>
       </c>
       <c r="D36" s="2" t="inlineStr">
         <is>
-          <t>입력과 차체 상태 정보가 100ms 기준으로 일관되게 반영된다</t>
+          <t>가속, 제동, 조향 입력이 100ms 기준으로 일관되게 반영되고 주행 판단 경로에 전달된다</t>
         </is>
       </c>
       <c r="E36" s="2" t="inlineStr"/>
@@ -24369,12 +24369,12 @@
       </c>
       <c r="C37" s="2" t="inlineStr">
         <is>
-          <t>비상등, 창문, 차체 편의 상태 통합 검증</t>
+          <t>비상등과 창문 상태 통합 검증</t>
         </is>
       </c>
       <c r="D37" s="2" t="inlineStr">
         <is>
-          <t>차체 제어 상태가 일관되게 유지된다</t>
+          <t>비상등과 창문 상태 변화가 누락 없이 반영된다</t>
         </is>
       </c>
       <c r="E37" s="2" t="inlineStr"/>
@@ -24444,12 +24444,12 @@
       </c>
       <c r="C40" s="2" t="inlineStr">
         <is>
-          <t>오디오, 음성 안내, TTS 상태 통합 검증</t>
+          <t>오디오 동시 실행 환경에서 경고 인지성 통합 검증</t>
         </is>
       </c>
       <c r="D40" s="2" t="inlineStr">
         <is>
-          <t>오디오와 음성 상태가 50/100ms 규칙을 만족하고 150ms 이내 HMI 정책에 반영된다</t>
+          <t>오디오 기능이 동시에 실행되는 상황에서도 경고 인지가 가능하고 관련 상태가 50/100ms 규칙을 만족하며 150ms 이내 HMI 정책에 반영된다</t>
         </is>
       </c>
       <c r="E40" s="2" t="inlineStr"/>
@@ -24464,17 +24464,17 @@
       </c>
       <c r="B41" s="2" t="inlineStr">
         <is>
-          <t>Req_078,Req_079</t>
+          <t>Req_078,Req_079,Req_081,Req_082</t>
         </is>
       </c>
       <c r="C41" s="2" t="inlineStr">
         <is>
-          <t>주요 출력 채널 가용성 및 대체 출력 통합 검증</t>
+          <t>주요 출력 채널 가용성, 팝업 과밀 억제, 대체 출력 통합 검증</t>
         </is>
       </c>
       <c r="D41" s="2" t="inlineStr">
         <is>
-          <t>출력 채널 상태 이상이 누락 없이 반영되고 대체 출력 전환 규칙이 150ms 내 충족된다</t>
+          <t>출력 채널 상태 이상이 누락 없이 반영되고 대체 출력 전환 규칙이 150ms 내 충족되며 비긴급 팝업 과밀이 억제되고 채널 불일치 시 동일 경고 맥락으로 복원된다</t>
         </is>
       </c>
       <c r="E41" s="2" t="inlineStr">
@@ -24493,7 +24493,7 @@
       </c>
       <c r="B42" s="2" t="inlineStr">
         <is>
-          <t>Req_071,Req_072,Req_073,Req_074</t>
+          <t>Req_070,Req_071,Req_072</t>
         </is>
       </c>
       <c r="C42" s="2" t="inlineStr">
@@ -24503,7 +24503,7 @@
       </c>
       <c r="D42" s="2" t="inlineStr">
         <is>
-          <t>접근거리 표시가 200ms 이내 갱신되고 경고 이력 조회 요청에 대한 응답이 누락 없이 반영된다</t>
+          <t>접근거리 표시가 200ms 이내 갱신되고 경고 이벤트가 공통 포맷으로 기록되며 경고 이력 조회 요청에 대한 응답이 누락 없이 반영된다</t>
         </is>
       </c>
       <c r="E42" s="2" t="inlineStr">
@@ -24672,12 +24672,12 @@
       </c>
       <c r="C48" s="2" t="inlineStr">
         <is>
-          <t>충전, 전력 변환, 구동 상태 통합 검증</t>
+          <t>충전, 전력 변환, 구동, 변속·열관리 상태 통합 검증</t>
         </is>
       </c>
       <c r="D48" s="2" t="inlineStr">
         <is>
-          <t>OBC, DCDC, MCU, INVERTER 상태가 100ms 주기로 반영되고 150ms 이내 구동 준비와 서비스 경고 맥락에 반영된다</t>
+          <t>OBC, DCDC, MCU, INVERTER와 변속·열관리 관련 상태가 100ms 주기로 반영되고 150ms 이내 구동 준비와 서비스 경고 맥락에 반영된다</t>
         </is>
       </c>
       <c r="E48" s="2" t="inlineStr">
@@ -24696,17 +24696,17 @@
       </c>
       <c r="B49" s="2" t="inlineStr">
         <is>
-          <t>Req_067,Req_068,Req_069,Req_070,Req_071,Req_072,Req_073,Req_074,Req_088,Req_089</t>
+          <t>Req_067,Req_069,Req_070,Req_073,Req_088,Req_089</t>
         </is>
       </c>
       <c r="C49" s="2" t="inlineStr">
         <is>
-          <t>표시 채널 출력 통합 검증</t>
+          <t>표시 채널 출력 및 서비스 상태 연계 통합 검증</t>
         </is>
       </c>
       <c r="D49" s="2" t="inlineStr">
         <is>
-          <t>경고 문구, 접근거리, 팝업, 테마, HUD 표시가 각 표시 채널에 일관되게 반영되고 채널 간 출력 차이는 50ms 이내이다</t>
+          <t>경고 문구와 접근거리 정보가 클러스터/HUD 등 표시 채널에 일관되게 반영되고 표시 방식 설정 및 표시·서비스 상태가 반영되며 채널 간 출력 차이는 50ms 이내이다</t>
         </is>
       </c>
       <c r="E49" s="2" t="inlineStr">
@@ -24725,17 +24725,17 @@
       </c>
       <c r="B50" s="2" t="inlineStr">
         <is>
-          <t>Req_044,Req_067,Req_068,Req_069,Req_070,Req_071,Req_072,Req_073,Req_074,Req_075,Req_076,Req_077,Req_078,Req_079,Req_080,Req_081,Req_082,Req_088,Req_089</t>
+          <t>Req_048,Req_074,Req_075,Req_076,Req_077,Req_080</t>
         </is>
       </c>
       <c r="C50" s="2" t="inlineStr">
         <is>
-          <t>오디오 안내 출력 통합 검증</t>
+          <t>오디오 안내 인지성과 입력 강건성 통합 검증</t>
         </is>
       </c>
       <c r="D50" s="2" t="inlineStr">
         <is>
-          <t>오디오 포커스, 음량, 음성안내, TTS 상태가 일관되게 반영되고 경합 시 150ms 이내 안내 정책이 안정화된다</t>
+          <t>음량 설정이 반영된 상태에서도 오디오 경합 상황에서 경고 인지가 가능하고 유효하지 않거나 stale한 입력은 판정에서 제외되며 동일 원인 경고 상태의 반복 진동이 억제된다</t>
         </is>
       </c>
       <c r="E50" s="2" t="inlineStr">
@@ -24754,7 +24754,7 @@
       </c>
       <c r="B51" s="2" t="inlineStr">
         <is>
-          <t>Req_120</t>
+          <t>Req_096</t>
         </is>
       </c>
       <c r="C51" s="2" t="inlineStr">
@@ -24783,7 +24783,7 @@
       </c>
       <c r="B52" s="2" t="inlineStr">
         <is>
-          <t>Req_121</t>
+          <t>Req_097</t>
         </is>
       </c>
       <c r="C52" s="2" t="inlineStr">
@@ -31647,7 +31647,7 @@
     <row r="112">
       <c r="A112" s="2" t="inlineStr">
         <is>
-          <t>Req_120</t>
+          <t>Req_096</t>
         </is>
       </c>
       <c r="B112" s="2" t="inlineStr">
@@ -31681,7 +31681,7 @@
     <row r="113">
       <c r="A113" s="2" t="inlineStr">
         <is>
-          <t>Req_121</t>
+          <t>Req_097</t>
         </is>
       </c>
       <c r="B113" s="2" t="inlineStr">
@@ -32150,7 +32150,7 @@
       </c>
       <c r="D142" s="2" t="inlineStr">
         <is>
-          <t>Req_002, Req_005, Req_008, Req_013, Req_014, Req_018, Req_019, Req_020, Req_025, Req_029, Req_030, Req_035, Req_036, Req_037, Req_038, Req_039, Req_040, Req_041, Req_044, Req_046, Req_047, Req_060, Req_063, Req_069, Req_070, Req_082, Req_083, Req_084, Req_085, Req_095, Req_120, Req_121</t>
+          <t>Req_002, Req_005, Req_008, Req_013, Req_014, Req_018, Req_019, Req_020, Req_025, Req_029, Req_030, Req_035, Req_036, Req_037, Req_038, Req_039, Req_040, Req_041, Req_044, Req_046, Req_047, Req_060, Req_063, Req_069, Req_070, Req_082, Req_083, Req_084, Req_085, Req_095, Req_096, Req_097</t>
         </is>
       </c>
       <c r="E142" s="2" t="n"/>

</xml_diff>

<commit_message>
docs(governance): update short paper package and assets
</commit_message>
<xml_diff>
--- a/driving-alert-workproducts/excel/submission_final_all_in_one.xlsx
+++ b/driving-alert-workproducts/excel/submission_final_all_in_one.xlsx
@@ -28647,7 +28647,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:K38"/>
+  <dimension ref="A1:K48"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="48" customWidth="1" min="1" max="1"/>
@@ -29661,6 +29661,160 @@
         </is>
       </c>
     </row>
+    <row r="39">
+      <c r="A39" s="2" t="n"/>
+      <c r="B39" s="2" t="n"/>
+      <c r="C39" s="2" t="n"/>
+      <c r="D39" s="2" t="n"/>
+      <c r="E39" s="2" t="n"/>
+      <c r="F39" s="2" t="n"/>
+      <c r="G39" s="2" t="n"/>
+      <c r="H39" s="2" t="n"/>
+      <c r="I39" s="2" t="n"/>
+      <c r="J39" s="2" t="n"/>
+      <c r="K39" s="2" t="n"/>
+    </row>
+    <row r="40">
+      <c r="A40" s="2" t="n"/>
+      <c r="B40" s="2" t="n"/>
+      <c r="C40" s="2" t="n"/>
+      <c r="D40" s="2" t="n"/>
+      <c r="E40" s="2" t="n"/>
+      <c r="F40" s="2" t="n"/>
+      <c r="G40" s="2" t="n"/>
+      <c r="H40" s="2" t="n"/>
+      <c r="I40" s="2" t="n"/>
+      <c r="J40" s="2" t="n"/>
+      <c r="K40" s="2" t="n"/>
+    </row>
+    <row r="41">
+      <c r="A41" s="1" t="inlineStr">
+        <is>
+          <t>연계 검증 문서</t>
+        </is>
+      </c>
+      <c r="B41" s="2" t="n"/>
+      <c r="C41" s="2" t="n"/>
+      <c r="D41" s="2" t="n"/>
+      <c r="E41" s="2" t="n"/>
+      <c r="F41" s="2" t="n"/>
+      <c r="G41" s="2" t="n"/>
+      <c r="H41" s="2" t="n"/>
+      <c r="I41" s="2" t="n"/>
+      <c r="J41" s="2" t="n"/>
+      <c r="K41" s="2" t="n"/>
+    </row>
+    <row r="42">
+      <c r="A42" s="2" t="n"/>
+      <c r="B42" s="2" t="n"/>
+      <c r="C42" s="2" t="n"/>
+      <c r="D42" s="2" t="n"/>
+      <c r="E42" s="2" t="n"/>
+      <c r="F42" s="2" t="n"/>
+      <c r="G42" s="2" t="n"/>
+      <c r="H42" s="2" t="n"/>
+      <c r="I42" s="2" t="n"/>
+      <c r="J42" s="2" t="n"/>
+      <c r="K42" s="2" t="n"/>
+    </row>
+    <row r="43">
+      <c r="A43" s="2" t="inlineStr">
+        <is>
+          <t>HARA의 안전 목표와 timing 가정은 아래 CANoe-side 검증 계약 문서와 함께 유지한다.</t>
+        </is>
+      </c>
+      <c r="B43" s="2" t="n"/>
+      <c r="C43" s="2" t="n"/>
+      <c r="D43" s="2" t="n"/>
+      <c r="E43" s="2" t="n"/>
+      <c r="F43" s="2" t="n"/>
+      <c r="G43" s="2" t="n"/>
+      <c r="H43" s="2" t="n"/>
+      <c r="I43" s="2" t="n"/>
+      <c r="J43" s="2" t="n"/>
+      <c r="K43" s="2" t="n"/>
+    </row>
+    <row r="44">
+      <c r="A44" s="2" t="n"/>
+      <c r="B44" s="2" t="n"/>
+      <c r="C44" s="2" t="n"/>
+      <c r="D44" s="2" t="n"/>
+      <c r="E44" s="2" t="n"/>
+      <c r="F44" s="2" t="n"/>
+      <c r="G44" s="2" t="n"/>
+      <c r="H44" s="2" t="n"/>
+      <c r="I44" s="2" t="n"/>
+      <c r="J44" s="2" t="n"/>
+      <c r="K44" s="2" t="n"/>
+    </row>
+    <row r="45">
+      <c r="A45" s="2" t="inlineStr">
+        <is>
+          <t>canoe/docs/verification/oracle.md</t>
+        </is>
+      </c>
+      <c r="B45" s="2" t="n"/>
+      <c r="C45" s="2" t="n"/>
+      <c r="D45" s="2" t="n"/>
+      <c r="E45" s="2" t="n"/>
+      <c r="F45" s="2" t="n"/>
+      <c r="G45" s="2" t="n"/>
+      <c r="H45" s="2" t="n"/>
+      <c r="I45" s="2" t="n"/>
+      <c r="J45" s="2" t="n"/>
+      <c r="K45" s="2" t="n"/>
+    </row>
+    <row r="46">
+      <c r="A46" s="2" t="inlineStr">
+        <is>
+          <t>canoe/docs/verification/acceptance-criteria.md</t>
+        </is>
+      </c>
+      <c r="B46" s="2" t="n"/>
+      <c r="C46" s="2" t="n"/>
+      <c r="D46" s="2" t="n"/>
+      <c r="E46" s="2" t="n"/>
+      <c r="F46" s="2" t="n"/>
+      <c r="G46" s="2" t="n"/>
+      <c r="H46" s="2" t="n"/>
+      <c r="I46" s="2" t="n"/>
+      <c r="J46" s="2" t="n"/>
+      <c r="K46" s="2" t="n"/>
+    </row>
+    <row r="47">
+      <c r="A47" s="2" t="inlineStr">
+        <is>
+          <t>canoe/docs/verification/test-asset-mapping.md</t>
+        </is>
+      </c>
+      <c r="B47" s="2" t="n"/>
+      <c r="C47" s="2" t="n"/>
+      <c r="D47" s="2" t="n"/>
+      <c r="E47" s="2" t="n"/>
+      <c r="F47" s="2" t="n"/>
+      <c r="G47" s="2" t="n"/>
+      <c r="H47" s="2" t="n"/>
+      <c r="I47" s="2" t="n"/>
+      <c r="J47" s="2" t="n"/>
+      <c r="K47" s="2" t="n"/>
+    </row>
+    <row r="48">
+      <c r="A48" s="2" t="inlineStr">
+        <is>
+          <t>canoe/docs/verification/execution-guide.md</t>
+        </is>
+      </c>
+      <c r="B48" s="2" t="n"/>
+      <c r="C48" s="2" t="n"/>
+      <c r="D48" s="2" t="n"/>
+      <c r="E48" s="2" t="n"/>
+      <c r="F48" s="2" t="n"/>
+      <c r="G48" s="2" t="n"/>
+      <c r="H48" s="2" t="n"/>
+      <c r="I48" s="2" t="n"/>
+      <c r="J48" s="2" t="n"/>
+      <c r="K48" s="2" t="n"/>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
@@ -29672,7 +29826,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C65"/>
+  <dimension ref="A1:C73"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="48" customWidth="1" min="1" max="1"/>
@@ -30364,6 +30518,66 @@
       </c>
       <c r="B65" s="2" t="n"/>
       <c r="C65" s="2" t="n"/>
+    </row>
+    <row r="66">
+      <c r="A66" s="2" t="n"/>
+      <c r="B66" s="2" t="n"/>
+      <c r="C66" s="2" t="n"/>
+    </row>
+    <row r="67">
+      <c r="A67" s="1" t="inlineStr">
+        <is>
+          <t>연계 계약 문서</t>
+        </is>
+      </c>
+      <c r="B67" s="2" t="n"/>
+      <c r="C67" s="2" t="n"/>
+    </row>
+    <row r="68">
+      <c r="A68" s="2" t="n"/>
+      <c r="B68" s="2" t="n"/>
+      <c r="C68" s="2" t="n"/>
+    </row>
+    <row r="69">
+      <c r="A69" s="2" t="inlineStr">
+        <is>
+          <t>ECU 표면 이름과 계층 표기는 아래 런타임 계약 문서와 함께 유지한다.</t>
+        </is>
+      </c>
+      <c r="B69" s="2" t="n"/>
+      <c r="C69" s="2" t="n"/>
+    </row>
+    <row r="70">
+      <c r="A70" s="2" t="n"/>
+      <c r="B70" s="2" t="n"/>
+      <c r="C70" s="2" t="n"/>
+    </row>
+    <row r="71">
+      <c r="A71" s="2" t="inlineStr">
+        <is>
+          <t>canoe/docs/contracts/communication-matrix.md</t>
+        </is>
+      </c>
+      <c r="B71" s="2" t="n"/>
+      <c r="C71" s="2" t="n"/>
+    </row>
+    <row r="72">
+      <c r="A72" s="2" t="inlineStr">
+        <is>
+          <t>canoe/docs/contracts/owner-route.md</t>
+        </is>
+      </c>
+      <c r="B72" s="2" t="n"/>
+      <c r="C72" s="2" t="n"/>
+    </row>
+    <row r="73">
+      <c r="A73" s="2" t="inlineStr">
+        <is>
+          <t>canoe/docs/contracts/layer-separation-policy.md</t>
+        </is>
+      </c>
+      <c r="B73" s="2" t="n"/>
+      <c r="C73" s="2" t="n"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
@@ -30376,7 +30590,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C86"/>
+  <dimension ref="A1:C95"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="48" customWidth="1" min="1" max="1"/>
@@ -31144,7 +31358,7 @@
     <row r="82">
       <c r="A82" s="1" t="inlineStr">
         <is>
-          <t>운영 메모</t>
+          <t>연계 인터페이스 문서</t>
         </is>
       </c>
       <c r="B82" s="2" t="n"/>
@@ -31158,29 +31372,98 @@
     <row r="84">
       <c r="A84" s="2" t="inlineStr">
         <is>
-          <t>제출 문서 기준에서는 현재 실행 중인 11-bit ID 체계를 사용한다.</t>
+          <t>CAN ID와 Ethernet/UDP 식별자 운용은 아래 문서와 함께 유지한다.</t>
         </is>
       </c>
       <c r="B84" s="2" t="n"/>
       <c r="C84" s="2" t="n"/>
     </row>
     <row r="85">
-      <c r="A85" s="2" t="inlineStr">
-        <is>
-          <t>29-bit 확장 정책은 진단 및 향후 확장 검토 항목으로 live SoT에서 별도로 관리한다.</t>
-        </is>
-      </c>
+      <c r="A85" s="2" t="n"/>
       <c r="B85" s="2" t="n"/>
       <c r="C85" s="2" t="n"/>
     </row>
     <row r="86">
       <c r="A86" s="2" t="inlineStr">
         <is>
-          <t>신규 메시지는 기존 활성 대역과 예약 구간 충돌 여부를 먼저 확인한다.</t>
+          <t>canoe/docs/contracts/communication-matrix.md</t>
         </is>
       </c>
       <c r="B86" s="2" t="n"/>
       <c r="C86" s="2" t="n"/>
+    </row>
+    <row r="87">
+      <c r="A87" s="2" t="inlineStr">
+        <is>
+          <t>canoe/docs/contracts/ethernet-interface.md</t>
+        </is>
+      </c>
+      <c r="B87" s="2" t="n"/>
+      <c r="C87" s="2" t="n"/>
+    </row>
+    <row r="88">
+      <c r="A88" s="2" t="inlineStr">
+        <is>
+          <t>canoe/docs/contracts/ethernet-backbone.md</t>
+        </is>
+      </c>
+      <c r="B88" s="2" t="n"/>
+      <c r="C88" s="2" t="n"/>
+    </row>
+    <row r="89">
+      <c r="A89" s="2" t="inlineStr">
+        <is>
+          <t>canoe/docs/contracts/multibus-policy.md</t>
+        </is>
+      </c>
+      <c r="B89" s="2" t="n"/>
+      <c r="C89" s="2" t="n"/>
+    </row>
+    <row r="90">
+      <c r="A90" s="2" t="n"/>
+      <c r="B90" s="2" t="n"/>
+      <c r="C90" s="2" t="n"/>
+    </row>
+    <row r="91">
+      <c r="A91" s="1" t="inlineStr">
+        <is>
+          <t>운영 메모</t>
+        </is>
+      </c>
+      <c r="B91" s="2" t="n"/>
+      <c r="C91" s="2" t="n"/>
+    </row>
+    <row r="92">
+      <c r="A92" s="2" t="n"/>
+      <c r="B92" s="2" t="n"/>
+      <c r="C92" s="2" t="n"/>
+    </row>
+    <row r="93">
+      <c r="A93" s="2" t="inlineStr">
+        <is>
+          <t>제출 문서 기준에서는 현재 실행 중인 11-bit ID 체계를 사용한다.</t>
+        </is>
+      </c>
+      <c r="B93" s="2" t="n"/>
+      <c r="C93" s="2" t="n"/>
+    </row>
+    <row r="94">
+      <c r="A94" s="2" t="inlineStr">
+        <is>
+          <t>29-bit 확장 정책은 진단 및 향후 확장 검토 항목으로 live SoT에서 별도로 관리한다.</t>
+        </is>
+      </c>
+      <c r="B94" s="2" t="n"/>
+      <c r="C94" s="2" t="n"/>
+    </row>
+    <row r="95">
+      <c r="A95" s="2" t="inlineStr">
+        <is>
+          <t>신규 메시지는 기존 활성 대역과 예약 구간 충돌 여부를 먼저 확인한다.</t>
+        </is>
+      </c>
+      <c r="B95" s="2" t="n"/>
+      <c r="C95" s="2" t="n"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>